<commit_message>
Se ajusto cada tarea a cada calendario
</commit_message>
<xml_diff>
--- a/Archivos/Archivos_origen/Planeación Doradobet El Salvador 2025.xlsx
+++ b/Archivos/Archivos_origen/Planeación Doradobet El Salvador 2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/jhor_caro_virtualsoft_tech/Documents/Documentos/GitHub/Planeaci-n_SEO/Archivos/Archivos_origen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="11_5760DF4CD5921C8A1011470F6B318B9F613A0262" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{28A7AFAF-48F9-4E9E-BE09-3DD61BD5D707}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="11_5760DF4CD5921C8A1011470F6B318B9F613A0262" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{665B7D72-E70C-4808-B02D-41C68A6EB32E}"/>
   <bookViews>
-    <workbookView xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Agosto" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="74">
   <si>
     <t>Blog/Plataforma</t>
   </si>
@@ -238,15 +238,6 @@
     <t>Tiempo estimado produccion</t>
   </si>
   <si>
-    <t>15 min</t>
-  </si>
-  <si>
-    <t>1 hora</t>
-  </si>
-  <si>
-    <t>30 min</t>
-  </si>
-  <si>
     <t>Juan Manuel</t>
   </si>
   <si>
@@ -416,7 +407,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -496,9 +487,13 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -514,6 +509,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -727,10 +726,12 @@
     <col min="5" max="9" width="26.6328125" customWidth="1"/>
     <col min="10" max="10" width="26.7265625" customWidth="1"/>
     <col min="11" max="11" width="26.6328125" customWidth="1"/>
-    <col min="12" max="14" width="13.26953125" customWidth="1"/>
+    <col min="12" max="13" width="13.26953125" customWidth="1"/>
+    <col min="14" max="14" width="13.26953125" style="35" customWidth="1"/>
     <col min="15" max="15" width="25.08984375" customWidth="1"/>
     <col min="16" max="17" width="27.7265625" customWidth="1"/>
-    <col min="18" max="20" width="14.453125" customWidth="1"/>
+    <col min="18" max="19" width="14.453125" customWidth="1"/>
+    <col min="20" max="20" width="14.453125" style="35" customWidth="1"/>
     <col min="21" max="21" width="23.90625" customWidth="1"/>
     <col min="22" max="22" width="31.90625" customWidth="1"/>
   </cols>
@@ -775,7 +776,7 @@
       <c r="M1" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="33" t="s">
         <v>69</v>
       </c>
       <c r="O1" s="3" t="s">
@@ -791,10 +792,10 @@
         <v>14</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>75</v>
+        <v>71</v>
+      </c>
+      <c r="T1" s="33" t="s">
+        <v>72</v>
       </c>
       <c r="U1" s="3" t="s">
         <v>15</v>
@@ -849,10 +850,10 @@
         <v>45875</v>
       </c>
       <c r="M2" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="N2" s="33" t="s">
         <v>70</v>
+      </c>
+      <c r="N2" s="34">
+        <v>15</v>
       </c>
       <c r="O2" s="13" t="s">
         <v>24</v>
@@ -862,10 +863,10 @@
         <v>45877</v>
       </c>
       <c r="S2" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="T2" s="33" t="s">
-        <v>70</v>
+        <v>73</v>
+      </c>
+      <c r="T2" s="34">
+        <v>15</v>
       </c>
       <c r="U2" s="14" t="s">
         <v>25</v>
@@ -904,10 +905,10 @@
         <v>45880</v>
       </c>
       <c r="M3" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="N3" s="33" t="s">
         <v>70</v>
+      </c>
+      <c r="N3" s="34">
+        <v>15</v>
       </c>
       <c r="O3" s="13" t="s">
         <v>26</v>
@@ -917,10 +918,10 @@
         <v>45880</v>
       </c>
       <c r="S3" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="T3" s="33" t="s">
-        <v>70</v>
+        <v>73</v>
+      </c>
+      <c r="T3" s="34">
+        <v>15</v>
       </c>
       <c r="U3" s="6" t="s">
         <v>31</v>
@@ -956,10 +957,10 @@
         <v>45888</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="N4" s="33" t="s">
-        <v>71</v>
+        <v>70</v>
+      </c>
+      <c r="N4" s="34">
+        <v>60</v>
       </c>
       <c r="O4" s="13" t="s">
         <v>37</v>
@@ -969,10 +970,10 @@
         <v>45889</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="T4" s="33" t="s">
-        <v>71</v>
+        <v>73</v>
+      </c>
+      <c r="T4" s="34">
+        <v>60</v>
       </c>
       <c r="U4" s="19"/>
       <c r="V4" s="14" t="s">
@@ -1007,10 +1008,10 @@
         <v>45897</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="N5" s="33" t="s">
-        <v>72</v>
+        <v>70</v>
+      </c>
+      <c r="N5" s="34">
+        <v>30</v>
       </c>
       <c r="O5" s="13" t="s">
         <v>39</v>
@@ -1020,10 +1021,10 @@
         <v>45898</v>
       </c>
       <c r="S5" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="T5" s="33" t="s">
-        <v>72</v>
+        <v>73</v>
+      </c>
+      <c r="T5" s="34">
+        <v>30</v>
       </c>
       <c r="U5" s="21" t="s">
         <v>42</v>
@@ -1045,12 +1046,12 @@
       <c r="K6" s="11"/>
       <c r="L6" s="12"/>
       <c r="M6" s="12"/>
-      <c r="N6" s="33"/>
+      <c r="N6" s="34"/>
       <c r="O6" s="19"/>
       <c r="P6" s="19"/>
       <c r="R6" s="12"/>
       <c r="S6" s="12"/>
-      <c r="T6" s="33"/>
+      <c r="T6" s="34"/>
       <c r="U6" s="19"/>
     </row>
     <row r="7" spans="1:38" ht="15.75" customHeight="1">
@@ -1067,13 +1068,13 @@
       <c r="K7" s="11"/>
       <c r="L7" s="12"/>
       <c r="M7" s="12"/>
-      <c r="N7" s="33"/>
+      <c r="N7" s="34"/>
       <c r="O7" s="24"/>
       <c r="P7" s="7"/>
       <c r="Q7" s="24"/>
       <c r="R7" s="12"/>
       <c r="S7" s="12"/>
-      <c r="T7" s="33"/>
+      <c r="T7" s="34"/>
       <c r="U7" s="19"/>
       <c r="V7" s="19"/>
     </row>
@@ -1089,13 +1090,13 @@
       <c r="K8" s="11"/>
       <c r="L8" s="12"/>
       <c r="M8" s="12"/>
-      <c r="N8" s="33"/>
+      <c r="N8" s="34"/>
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
       <c r="Q8" s="24"/>
       <c r="R8" s="12"/>
       <c r="S8" s="12"/>
-      <c r="T8" s="33"/>
+      <c r="T8" s="34"/>
       <c r="U8" s="10"/>
       <c r="V8" s="19"/>
     </row>
@@ -1112,13 +1113,13 @@
       <c r="K9" s="11"/>
       <c r="L9" s="12"/>
       <c r="M9" s="12"/>
-      <c r="N9" s="33"/>
+      <c r="N9" s="34"/>
       <c r="O9" s="24"/>
       <c r="P9" s="7"/>
       <c r="Q9" s="24"/>
       <c r="R9" s="12"/>
       <c r="S9" s="12"/>
-      <c r="T9" s="33"/>
+      <c r="T9" s="34"/>
       <c r="U9" s="19"/>
       <c r="V9" s="19"/>
     </row>
@@ -1134,13 +1135,13 @@
       <c r="K10" s="11"/>
       <c r="L10" s="12"/>
       <c r="M10" s="12"/>
-      <c r="N10" s="33"/>
+      <c r="N10" s="34"/>
       <c r="O10" s="24"/>
       <c r="P10" s="7"/>
       <c r="Q10" s="24"/>
       <c r="R10" s="12"/>
       <c r="S10" s="12"/>
-      <c r="T10" s="33"/>
+      <c r="T10" s="34"/>
       <c r="U10" s="19"/>
     </row>
     <row r="11" spans="1:38" ht="15.75" customHeight="1">
@@ -1153,11 +1154,11 @@
       <c r="K11" s="8"/>
       <c r="L11" s="12"/>
       <c r="M11" s="12"/>
-      <c r="N11" s="33"/>
+      <c r="N11" s="34"/>
       <c r="O11" s="19"/>
       <c r="R11" s="26"/>
       <c r="S11" s="12"/>
-      <c r="T11" s="33"/>
+      <c r="T11" s="34"/>
     </row>
     <row r="12" spans="1:38" ht="15.75" customHeight="1">
       <c r="A12" s="15"/>
@@ -1173,13 +1174,13 @@
       <c r="K12" s="11"/>
       <c r="L12" s="12"/>
       <c r="M12" s="12"/>
-      <c r="N12" s="33"/>
+      <c r="N12" s="34"/>
       <c r="O12" s="10"/>
       <c r="P12" s="19"/>
       <c r="Q12" s="19"/>
       <c r="R12" s="12"/>
       <c r="S12" s="12"/>
-      <c r="T12" s="33"/>
+      <c r="T12" s="34"/>
       <c r="U12" s="19"/>
       <c r="V12" s="19"/>
     </row>
@@ -1197,13 +1198,13 @@
       <c r="K13" s="11"/>
       <c r="L13" s="12"/>
       <c r="M13" s="12"/>
-      <c r="N13" s="33"/>
+      <c r="N13" s="34"/>
       <c r="O13" s="11"/>
       <c r="P13" s="10"/>
       <c r="Q13" s="10"/>
       <c r="R13" s="12"/>
       <c r="S13" s="12"/>
-      <c r="T13" s="33"/>
+      <c r="T13" s="34"/>
       <c r="U13" s="10"/>
       <c r="V13" s="10"/>
     </row>
@@ -1219,13 +1220,13 @@
       <c r="K14" s="11"/>
       <c r="L14" s="12"/>
       <c r="M14" s="12"/>
-      <c r="N14" s="33"/>
+      <c r="N14" s="34"/>
       <c r="O14" s="24"/>
       <c r="P14" s="10"/>
       <c r="Q14" s="24"/>
       <c r="R14" s="12"/>
       <c r="S14" s="12"/>
-      <c r="T14" s="33"/>
+      <c r="T14" s="34"/>
       <c r="U14" s="19"/>
       <c r="V14" s="19"/>
     </row>
@@ -1239,11 +1240,11 @@
       <c r="K15" s="8"/>
       <c r="L15" s="12"/>
       <c r="M15" s="12"/>
-      <c r="N15" s="33"/>
+      <c r="N15" s="34"/>
       <c r="O15" s="19"/>
       <c r="R15" s="26"/>
       <c r="S15" s="12"/>
-      <c r="T15" s="33"/>
+      <c r="T15" s="34"/>
       <c r="V15" s="19"/>
     </row>
     <row r="16" spans="1:38" ht="15.75" customHeight="1">
@@ -1252,10 +1253,10 @@
       <c r="J16" s="11"/>
       <c r="K16" s="19"/>
       <c r="M16" s="12"/>
-      <c r="N16" s="33"/>
+      <c r="N16" s="34"/>
       <c r="O16" s="19"/>
       <c r="S16" s="12"/>
-      <c r="T16" s="33"/>
+      <c r="T16" s="34"/>
     </row>
     <row r="17" spans="2:22" ht="15.75" customHeight="1">
       <c r="B17" s="6"/>
@@ -1267,10 +1268,10 @@
       <c r="J17" s="11"/>
       <c r="K17" s="19"/>
       <c r="M17" s="12"/>
-      <c r="N17" s="33"/>
+      <c r="N17" s="34"/>
       <c r="O17" s="19"/>
       <c r="S17" s="12"/>
-      <c r="T17" s="33"/>
+      <c r="T17" s="34"/>
     </row>
     <row r="18" spans="2:22" ht="15.75" customHeight="1">
       <c r="C18" s="7"/>
@@ -1281,10 +1282,10 @@
       <c r="J18" s="11"/>
       <c r="K18" s="19"/>
       <c r="M18" s="12"/>
-      <c r="N18" s="33"/>
+      <c r="N18" s="34"/>
       <c r="O18" s="19"/>
       <c r="S18" s="12"/>
-      <c r="T18" s="33"/>
+      <c r="T18" s="34"/>
       <c r="V18" s="19"/>
     </row>
     <row r="19" spans="2:22" ht="15.75" customHeight="1">
@@ -8131,10 +8132,12 @@
     <col min="5" max="9" width="26.6328125" customWidth="1"/>
     <col min="10" max="10" width="26.7265625" customWidth="1"/>
     <col min="11" max="11" width="26.6328125" customWidth="1"/>
-    <col min="12" max="14" width="13.26953125" customWidth="1"/>
+    <col min="12" max="13" width="13.26953125" customWidth="1"/>
+    <col min="14" max="14" width="13.26953125" style="35" customWidth="1"/>
     <col min="15" max="15" width="25.08984375" customWidth="1"/>
     <col min="16" max="17" width="27.7265625" customWidth="1"/>
-    <col min="18" max="20" width="14.453125" customWidth="1"/>
+    <col min="18" max="19" width="14.453125" customWidth="1"/>
+    <col min="20" max="20" width="14.453125" style="35" customWidth="1"/>
     <col min="21" max="21" width="23.90625" customWidth="1"/>
     <col min="22" max="22" width="31.90625" customWidth="1"/>
   </cols>
@@ -8179,7 +8182,7 @@
       <c r="M1" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="33" t="s">
         <v>69</v>
       </c>
       <c r="O1" s="3" t="s">
@@ -8195,10 +8198,10 @@
         <v>14</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>75</v>
+        <v>71</v>
+      </c>
+      <c r="T1" s="33" t="s">
+        <v>72</v>
       </c>
       <c r="U1" s="3" t="s">
         <v>15</v>
@@ -8254,10 +8257,10 @@
         <v>45898</v>
       </c>
       <c r="M2" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="N2" s="33" t="s">
         <v>70</v>
+      </c>
+      <c r="N2" s="34">
+        <v>15</v>
       </c>
       <c r="O2" s="28" t="s">
         <v>44</v>
@@ -8268,10 +8271,10 @@
         <v>45901</v>
       </c>
       <c r="S2" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="T2" s="33" t="s">
-        <v>70</v>
+        <v>73</v>
+      </c>
+      <c r="T2" s="34">
+        <v>15</v>
       </c>
       <c r="U2" s="27" t="s">
         <v>43</v>
@@ -8310,10 +8313,10 @@
         <v>45903</v>
       </c>
       <c r="M3" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="N3" s="33" t="s">
         <v>70</v>
+      </c>
+      <c r="N3" s="34">
+        <v>15</v>
       </c>
       <c r="O3" s="30" t="s">
         <v>50</v>
@@ -8324,10 +8327,10 @@
         <v>45910</v>
       </c>
       <c r="S3" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="T3" s="33" t="s">
-        <v>70</v>
+        <v>73</v>
+      </c>
+      <c r="T3" s="34">
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:38" ht="37.5">
@@ -8362,10 +8365,10 @@
         <v>45904</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="N4" s="33" t="s">
-        <v>71</v>
+        <v>70</v>
+      </c>
+      <c r="N4" s="34">
+        <v>60</v>
       </c>
       <c r="O4" s="30" t="s">
         <v>61</v>
@@ -8376,10 +8379,10 @@
         <v>45922</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="T4" s="33" t="s">
-        <v>71</v>
+        <v>73</v>
+      </c>
+      <c r="T4" s="34">
+        <v>60</v>
       </c>
       <c r="U4" s="19"/>
       <c r="V4" s="19"/>
@@ -8414,10 +8417,10 @@
         <v>45905</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="N5" s="33" t="s">
-        <v>72</v>
+        <v>70</v>
+      </c>
+      <c r="N5" s="34">
+        <v>30</v>
       </c>
       <c r="O5" s="24"/>
       <c r="P5" s="24"/>
@@ -8426,10 +8429,10 @@
         <v>45930</v>
       </c>
       <c r="S5" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="T5" s="33" t="s">
-        <v>72</v>
+        <v>73</v>
+      </c>
+      <c r="T5" s="34">
+        <v>30</v>
       </c>
       <c r="V5" s="19"/>
     </row>
@@ -8446,12 +8449,12 @@
       <c r="K6" s="11"/>
       <c r="L6" s="12"/>
       <c r="M6" s="12"/>
-      <c r="N6" s="33"/>
+      <c r="N6" s="34"/>
       <c r="O6" s="19"/>
       <c r="P6" s="19"/>
       <c r="R6" s="12"/>
       <c r="S6" s="12"/>
-      <c r="T6" s="33"/>
+      <c r="T6" s="34"/>
       <c r="U6" s="19"/>
     </row>
     <row r="7" spans="1:38">
@@ -8468,13 +8471,13 @@
       <c r="K7" s="11"/>
       <c r="L7" s="12"/>
       <c r="M7" s="12"/>
-      <c r="N7" s="33"/>
+      <c r="N7" s="34"/>
       <c r="O7" s="24"/>
       <c r="P7" s="7"/>
       <c r="Q7" s="24"/>
       <c r="R7" s="12"/>
       <c r="S7" s="12"/>
-      <c r="T7" s="33"/>
+      <c r="T7" s="34"/>
       <c r="U7" s="19"/>
       <c r="V7" s="19"/>
     </row>
@@ -8490,13 +8493,13 @@
       <c r="K8" s="11"/>
       <c r="L8" s="12"/>
       <c r="M8" s="12"/>
-      <c r="N8" s="33"/>
+      <c r="N8" s="34"/>
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
       <c r="Q8" s="24"/>
       <c r="R8" s="12"/>
       <c r="S8" s="12"/>
-      <c r="T8" s="33"/>
+      <c r="T8" s="34"/>
       <c r="U8" s="10"/>
       <c r="V8" s="19"/>
     </row>
@@ -8513,13 +8516,13 @@
       <c r="K9" s="11"/>
       <c r="L9" s="12"/>
       <c r="M9" s="12"/>
-      <c r="N9" s="33"/>
+      <c r="N9" s="34"/>
       <c r="O9" s="24"/>
       <c r="P9" s="7"/>
       <c r="Q9" s="24"/>
       <c r="R9" s="12"/>
       <c r="S9" s="12"/>
-      <c r="T9" s="33"/>
+      <c r="T9" s="34"/>
       <c r="U9" s="19"/>
       <c r="V9" s="19"/>
     </row>
@@ -8535,13 +8538,13 @@
       <c r="K10" s="11"/>
       <c r="L10" s="12"/>
       <c r="M10" s="12"/>
-      <c r="N10" s="33"/>
+      <c r="N10" s="34"/>
       <c r="O10" s="24"/>
       <c r="P10" s="7"/>
       <c r="Q10" s="24"/>
       <c r="R10" s="12"/>
       <c r="S10" s="12"/>
-      <c r="T10" s="33"/>
+      <c r="T10" s="34"/>
       <c r="U10" s="19"/>
     </row>
     <row r="11" spans="1:38">
@@ -8554,11 +8557,11 @@
       <c r="K11" s="8"/>
       <c r="L11" s="12"/>
       <c r="M11" s="12"/>
-      <c r="N11" s="33"/>
+      <c r="N11" s="34"/>
       <c r="O11" s="19"/>
       <c r="R11" s="26"/>
       <c r="S11" s="12"/>
-      <c r="T11" s="33"/>
+      <c r="T11" s="34"/>
     </row>
     <row r="12" spans="1:38">
       <c r="A12" s="15"/>
@@ -8574,13 +8577,13 @@
       <c r="K12" s="11"/>
       <c r="L12" s="12"/>
       <c r="M12" s="12"/>
-      <c r="N12" s="33"/>
+      <c r="N12" s="34"/>
       <c r="O12" s="10"/>
       <c r="P12" s="19"/>
       <c r="Q12" s="19"/>
       <c r="R12" s="12"/>
       <c r="S12" s="12"/>
-      <c r="T12" s="33"/>
+      <c r="T12" s="34"/>
       <c r="U12" s="19"/>
       <c r="V12" s="19"/>
     </row>
@@ -8598,13 +8601,13 @@
       <c r="K13" s="11"/>
       <c r="L13" s="12"/>
       <c r="M13" s="12"/>
-      <c r="N13" s="33"/>
+      <c r="N13" s="34"/>
       <c r="O13" s="11"/>
       <c r="P13" s="10"/>
       <c r="Q13" s="10"/>
       <c r="R13" s="12"/>
       <c r="S13" s="12"/>
-      <c r="T13" s="33"/>
+      <c r="T13" s="34"/>
       <c r="U13" s="10"/>
       <c r="V13" s="10"/>
     </row>
@@ -8620,13 +8623,13 @@
       <c r="K14" s="11"/>
       <c r="L14" s="12"/>
       <c r="M14" s="12"/>
-      <c r="N14" s="33"/>
+      <c r="N14" s="34"/>
       <c r="O14" s="24"/>
       <c r="P14" s="10"/>
       <c r="Q14" s="24"/>
       <c r="R14" s="12"/>
       <c r="S14" s="12"/>
-      <c r="T14" s="33"/>
+      <c r="T14" s="34"/>
       <c r="U14" s="19"/>
       <c r="V14" s="19"/>
     </row>
@@ -8640,11 +8643,11 @@
       <c r="K15" s="8"/>
       <c r="L15" s="12"/>
       <c r="M15" s="12"/>
-      <c r="N15" s="33"/>
+      <c r="N15" s="34"/>
       <c r="O15" s="19"/>
       <c r="R15" s="26"/>
       <c r="S15" s="12"/>
-      <c r="T15" s="33"/>
+      <c r="T15" s="34"/>
       <c r="V15" s="19"/>
     </row>
     <row r="16" spans="1:38">
@@ -8653,10 +8656,10 @@
       <c r="J16" s="11"/>
       <c r="K16" s="19"/>
       <c r="M16" s="12"/>
-      <c r="N16" s="33"/>
+      <c r="N16" s="34"/>
       <c r="O16" s="19"/>
       <c r="S16" s="12"/>
-      <c r="T16" s="33"/>
+      <c r="T16" s="34"/>
     </row>
     <row r="17" spans="2:22">
       <c r="B17" s="6"/>
@@ -8668,10 +8671,10 @@
       <c r="J17" s="11"/>
       <c r="K17" s="19"/>
       <c r="M17" s="12"/>
-      <c r="N17" s="33"/>
+      <c r="N17" s="34"/>
       <c r="O17" s="19"/>
       <c r="S17" s="12"/>
-      <c r="T17" s="33"/>
+      <c r="T17" s="34"/>
     </row>
     <row r="18" spans="2:22">
       <c r="C18" s="7"/>
@@ -8682,10 +8685,10 @@
       <c r="J18" s="11"/>
       <c r="K18" s="19"/>
       <c r="M18" s="12"/>
-      <c r="N18" s="33"/>
+      <c r="N18" s="34"/>
       <c r="O18" s="19"/>
       <c r="S18" s="12"/>
-      <c r="T18" s="33"/>
+      <c r="T18" s="34"/>
       <c r="V18" s="19"/>
     </row>
     <row r="19" spans="2:22">

</xml_diff>